<commit_message>
fix(phase7): Update BASE_URL default to live GitHub Pages and ensure 100% test pass rate
</commit_message>
<xml_diff>
--- a/automation/reports/Excel/Automation_Test_Report.xlsx
+++ b/automation/reports/Excel/Automation_Test_Report.xlsx
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.862</v>
+        <v>2.541</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.021</v>
+        <v>0.03</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.017</v>
+        <v>0.028</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.016</v>
+        <v>0.019</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.017</v>
+        <v>0.02</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.017</v>
+        <v>0.022</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.017</v>
+        <v>0.019</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.016</v>
+        <v>0.021</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.015</v>
+        <v>0.02</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.015</v>
+        <v>0.019</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.015</v>
+        <v>0.022</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1899,7 +1899,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.134</v>
+        <v>0.233</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2364,7 +2364,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>0.017</v>
+        <v>0.025</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>0.016</v>
+        <v>0.023</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>0.241</v>
+        <v>1.262</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -3759,7 +3759,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>0.033</v>
+        <v>0.044</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -4224,7 +4224,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>0.017</v>
+        <v>0.021</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -4689,7 +4689,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>0.015</v>
+        <v>0.024</v>
       </c>
       <c r="F137" t="inlineStr">
         <is>
@@ -5154,7 +5154,7 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>0.015</v>
+        <v>0.027</v>
       </c>
       <c r="F152" t="inlineStr">
         <is>
@@ -5619,7 +5619,7 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>0.015</v>
+        <v>0.02</v>
       </c>
       <c r="F167" t="inlineStr">
         <is>
@@ -6084,7 +6084,7 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>0.015</v>
+        <v>0.02</v>
       </c>
       <c r="F182" t="inlineStr">
         <is>
@@ -6549,7 +6549,7 @@
         </is>
       </c>
       <c r="E197" t="n">
-        <v>0.015</v>
+        <v>0.017</v>
       </c>
       <c r="F197" t="inlineStr">
         <is>
@@ -7014,7 +7014,7 @@
         </is>
       </c>
       <c r="E212" t="n">
-        <v>0.026</v>
+        <v>0.033</v>
       </c>
       <c r="F212" t="inlineStr">
         <is>
@@ -7479,7 +7479,7 @@
         </is>
       </c>
       <c r="E227" t="n">
-        <v>0.02</v>
+        <v>0.025</v>
       </c>
       <c r="F227" t="inlineStr">
         <is>
@@ -7944,7 +7944,7 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>0.023</v>
+        <v>0.032</v>
       </c>
       <c r="F242" t="inlineStr">
         <is>
@@ -8409,7 +8409,7 @@
         </is>
       </c>
       <c r="E257" t="n">
-        <v>0.02</v>
+        <v>0.038</v>
       </c>
       <c r="F257" t="inlineStr">
         <is>
@@ -8874,7 +8874,7 @@
         </is>
       </c>
       <c r="E272" t="n">
-        <v>0.016</v>
+        <v>0.03</v>
       </c>
       <c r="F272" t="inlineStr">
         <is>
@@ -9339,7 +9339,7 @@
         </is>
       </c>
       <c r="E287" t="n">
-        <v>0.015</v>
+        <v>0.033</v>
       </c>
       <c r="F287" t="inlineStr">
         <is>
@@ -9804,7 +9804,7 @@
         </is>
       </c>
       <c r="E302" t="n">
-        <v>0.017</v>
+        <v>0.038</v>
       </c>
       <c r="F302" t="inlineStr">
         <is>
@@ -10269,7 +10269,7 @@
         </is>
       </c>
       <c r="E317" t="n">
-        <v>0.021</v>
+        <v>0.036</v>
       </c>
       <c r="F317" t="inlineStr">
         <is>
@@ -10734,7 +10734,7 @@
         </is>
       </c>
       <c r="E332" t="n">
-        <v>0.017</v>
+        <v>0.025</v>
       </c>
       <c r="F332" t="inlineStr">
         <is>
@@ -11199,7 +11199,7 @@
         </is>
       </c>
       <c r="E347" t="n">
-        <v>0.015</v>
+        <v>0.035</v>
       </c>
       <c r="F347" t="inlineStr">
         <is>
@@ -11664,7 +11664,7 @@
         </is>
       </c>
       <c r="E362" t="n">
-        <v>0.02</v>
+        <v>0.035</v>
       </c>
       <c r="F362" t="inlineStr">
         <is>
@@ -12129,7 +12129,7 @@
         </is>
       </c>
       <c r="E377" t="n">
-        <v>0.015</v>
+        <v>0.052</v>
       </c>
       <c r="F377" t="inlineStr">
         <is>
@@ -12594,7 +12594,7 @@
         </is>
       </c>
       <c r="E392" t="n">
-        <v>0.015</v>
+        <v>0.045</v>
       </c>
       <c r="F392" t="inlineStr">
         <is>
@@ -13059,7 +13059,7 @@
         </is>
       </c>
       <c r="E407" t="n">
-        <v>0.015</v>
+        <v>0.034</v>
       </c>
       <c r="F407" t="inlineStr">
         <is>
@@ -13524,7 +13524,7 @@
         </is>
       </c>
       <c r="E422" t="n">
-        <v>0.016</v>
+        <v>0.033</v>
       </c>
       <c r="F422" t="inlineStr">
         <is>
@@ -13989,7 +13989,7 @@
         </is>
       </c>
       <c r="E437" t="n">
-        <v>0.016</v>
+        <v>0.03</v>
       </c>
       <c r="F437" t="inlineStr">
         <is>
@@ -14454,7 +14454,7 @@
         </is>
       </c>
       <c r="E452" t="n">
-        <v>0.015</v>
+        <v>0.032</v>
       </c>
       <c r="F452" t="inlineStr">
         <is>
@@ -14919,7 +14919,7 @@
         </is>
       </c>
       <c r="E467" t="n">
-        <v>0.016</v>
+        <v>0.031</v>
       </c>
       <c r="F467" t="inlineStr">
         <is>
@@ -15117,7 +15117,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.862</v>
+        <v>2.541</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -15142,7 +15142,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.021</v>
+        <v>0.03</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -15167,7 +15167,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.017</v>
+        <v>0.028</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -15192,7 +15192,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.016</v>
+        <v>0.019</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -15217,7 +15217,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.017</v>
+        <v>0.02</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -15242,7 +15242,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.017</v>
+        <v>0.022</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -15267,7 +15267,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.017</v>
+        <v>0.019</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -15292,7 +15292,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.016</v>
+        <v>0.021</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -15317,7 +15317,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.015</v>
+        <v>0.02</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -15342,7 +15342,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.015</v>
+        <v>0.019</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -15492,7 +15492,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.015</v>
+        <v>0.022</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -15867,7 +15867,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -16242,7 +16242,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.134</v>
+        <v>0.233</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -16617,7 +16617,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.017</v>
+        <v>0.025</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -16992,7 +16992,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.016</v>
+        <v>0.023</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -17367,7 +17367,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>0.241</v>
+        <v>1.262</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -17742,7 +17742,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.033</v>
+        <v>0.044</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -18117,7 +18117,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>0.017</v>
+        <v>0.021</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -18492,7 +18492,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>0.015</v>
+        <v>0.024</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -18867,7 +18867,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>0.015</v>
+        <v>0.027</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -19242,7 +19242,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>0.015</v>
+        <v>0.02</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -19617,7 +19617,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>0.015</v>
+        <v>0.02</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -19992,7 +19992,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>0.015</v>
+        <v>0.017</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -20367,7 +20367,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>0.026</v>
+        <v>0.033</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -20742,7 +20742,7 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>0.02</v>
+        <v>0.025</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -21117,7 +21117,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>0.023</v>
+        <v>0.032</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -21492,7 +21492,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>0.02</v>
+        <v>0.038</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -21867,7 +21867,7 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>0.016</v>
+        <v>0.03</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -22242,7 +22242,7 @@
         </is>
       </c>
       <c r="D287" t="n">
-        <v>0.015</v>
+        <v>0.033</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -22617,7 +22617,7 @@
         </is>
       </c>
       <c r="D302" t="n">
-        <v>0.017</v>
+        <v>0.038</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -22992,7 +22992,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>0.021</v>
+        <v>0.036</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -23367,7 +23367,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>0.017</v>
+        <v>0.025</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -23742,7 +23742,7 @@
         </is>
       </c>
       <c r="D347" t="n">
-        <v>0.015</v>
+        <v>0.035</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -24117,7 +24117,7 @@
         </is>
       </c>
       <c r="D362" t="n">
-        <v>0.02</v>
+        <v>0.035</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -24492,7 +24492,7 @@
         </is>
       </c>
       <c r="D377" t="n">
-        <v>0.015</v>
+        <v>0.052</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -24867,7 +24867,7 @@
         </is>
       </c>
       <c r="D392" t="n">
-        <v>0.015</v>
+        <v>0.045</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -25242,7 +25242,7 @@
         </is>
       </c>
       <c r="D407" t="n">
-        <v>0.015</v>
+        <v>0.034</v>
       </c>
       <c r="E407" t="inlineStr">
         <is>
@@ -25617,7 +25617,7 @@
         </is>
       </c>
       <c r="D422" t="n">
-        <v>0.016</v>
+        <v>0.033</v>
       </c>
       <c r="E422" t="inlineStr">
         <is>
@@ -25992,7 +25992,7 @@
         </is>
       </c>
       <c r="D437" t="n">
-        <v>0.016</v>
+        <v>0.03</v>
       </c>
       <c r="E437" t="inlineStr">
         <is>
@@ -26367,7 +26367,7 @@
         </is>
       </c>
       <c r="D452" t="n">
-        <v>0.015</v>
+        <v>0.032</v>
       </c>
       <c r="E452" t="inlineStr">
         <is>
@@ -26742,7 +26742,7 @@
         </is>
       </c>
       <c r="D467" t="n">
-        <v>0.016</v>
+        <v>0.031</v>
       </c>
       <c r="E467" t="inlineStr">
         <is>
@@ -27041,7 +27041,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.88</v>
+        <v>5.11</v>
       </c>
     </row>
     <row r="8">

</xml_diff>